<commit_message>
Fix text wrapping and column width for output cells in Standalone Tool
</commit_message>
<xml_diff>
--- a/Standalone_Cable_Routing_Tool.xlsx
+++ b/Standalone_Cable_Routing_Tool.xlsx
@@ -198,7 +198,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -234,6 +234,17 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -637,11 +648,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30" customWidth="1" style="13" min="1" max="1"/>
-    <col width="34" customWidth="1" style="13" min="2" max="2"/>
+    <col width="65" customWidth="1" style="13" min="2" max="2"/>
     <col width="24" customWidth="1" style="13" min="3" max="3"/>
     <col hidden="1" width="24" customWidth="1" style="13" min="4" max="5"/>
     <col width="24" customWidth="1" style="13" min="6" max="7"/>
@@ -672,7 +683,7 @@
           <t>Area</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>Outdoor</t>
         </is>
@@ -693,7 +704,7 @@
           <t>Primary System Type</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Power 400/230V</t>
         </is>
@@ -714,7 +725,7 @@
           <t>Shared With System Type</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="19" t="inlineStr">
         <is>
           <t>Speaker 100V</t>
         </is>
@@ -735,7 +746,7 @@
           <t>Same Tray Considered</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -756,7 +767,7 @@
           <t>Separator Applied</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -777,7 +788,7 @@
           <t>Construction Schedule</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>Different Phase</t>
         </is>
@@ -798,7 +809,7 @@
           <t>Tray Spare Percentage</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="20" t="n">
         <v>0.2</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -817,7 +828,7 @@
           <t>Owner Approval Granted?</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -838,7 +849,7 @@
           <t>Automatic Decision Output</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
@@ -848,7 +859,7 @@
         <v/>
       </c>
     </row>
-    <row r="13">
+    <row r="13" s="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Sharing Allowed</t>
@@ -859,7 +870,7 @@
         <v/>
       </c>
     </row>
-    <row r="14">
+    <row r="14" s="13">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Separator Mandatory</t>
@@ -870,7 +881,7 @@
         <v/>
       </c>
     </row>
-    <row r="15">
+    <row r="15" s="13">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Dedicated Tray Required</t>
@@ -881,7 +892,7 @@
         <v/>
       </c>
     </row>
-    <row r="16">
+    <row r="16" s="13">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Separation Review Required</t>
@@ -892,7 +903,7 @@
         <v/>
       </c>
     </row>
-    <row r="17">
+    <row r="17" s="13">
       <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Construction Schedule Compatible</t>
@@ -903,7 +914,7 @@
         <v/>
       </c>
     </row>
-    <row r="18">
+    <row r="18" s="13">
       <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Tray Spare Status</t>
@@ -914,7 +925,7 @@
         <v/>
       </c>
     </row>
-    <row r="19">
+    <row r="19" s="13">
       <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Typical Route Model</t>
@@ -925,7 +936,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="45" customHeight="1" s="13">
+    <row r="20" s="13">
       <c r="A20" s="7" t="inlineStr">
         <is>
           <t>Final Decision Owner</t>
@@ -936,7 +947,7 @@
         <v/>
       </c>
     </row>
-    <row r="21">
+    <row r="21" s="13">
       <c r="A21" s="7" t="inlineStr">
         <is>
           <t>Layout Strategy</t>
@@ -947,7 +958,7 @@
         <v/>
       </c>
     </row>
-    <row r="22">
+    <row r="22" s="13">
       <c r="A22" s="7" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -958,10 +969,10 @@
         <v/>
       </c>
     </row>
-    <row r="23">
+    <row r="23" s="13">
       <c r="A23" s="12" t="n"/>
     </row>
-    <row r="24">
+    <row r="24" s="13">
       <c r="A24" s="1" t="inlineStr">
         <is>
           <t>Owner Discussion Notes</t>
@@ -983,6 +994,10 @@
       <c r="D25" s="17" t="n"/>
       <c r="E25" s="18" t="n"/>
     </row>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Fix ExcelJS parsing crash by clearing Table metadata from template and update standalone HTML
</commit_message>
<xml_diff>
--- a/Standalone_Cable_Routing_Tool.xlsx
+++ b/Standalone_Cable_Routing_Tool.xlsx
@@ -343,20 +343,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TypicalRouteModels" displayName="TypicalRouteModels" ref="A1:E5" headerRowCount="1">
-  <autoFilter ref="A1:E5"/>
-  <tableColumns count="5">
-    <tableColumn id="1" name="Route Code"/>
-    <tableColumn id="2" name="Area"/>
-    <tableColumn id="3" name="Typical Route Model"/>
-    <tableColumn id="4" name="Default Owner"/>
-    <tableColumn id="5" name="Description"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -648,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30" customWidth="1" style="13" min="1" max="1"/>
@@ -994,10 +980,6 @@
       <c r="D25" s="17" t="n"/>
       <c r="E25" s="18" t="n"/>
     </row>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="3">
@@ -1756,8 +1738,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>